<commit_message>
test: casos y testing exploratorio del sprint 3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/casos-de-prueba.xlsx
+++ b/docs/testing/casos-de-prueba.xlsx
@@ -140,7 +140,7 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-15 12:24:08</t>
+          <t xml:space="preserve">2026-10-15 12:35:33</t>
         </is>
       </c>
     </row>
@@ -353,42 +353,58 @@
         </is>
       </c>
       <c r="B25" s="8">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C25" s="8">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D25" s="8">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Criterios</t>
-        </is>
-      </c>
-    </row>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 3</t>
+        </is>
+      </c>
+      <c r="B26" s="8">
+        <v>21</v>
+      </c>
+      <c r="C26" s="8">
+        <v>21</v>
+      </c>
+      <c r="D26" s="8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smoke</t>
-        </is>
-      </c>
-      <c r="B28" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Camino feliz de cada historia y verificaciones mínimas de seguridad e infraestructura. Si falla, el build no es apto para seguir probando.</t>
+          <t xml:space="preserve">Criterios</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Smoke</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Camino feliz de cada historia y verificaciones mínimas de seguridad e infraestructura. Si falla, el build no es apto para seguir probando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Regresión</t>
         </is>
       </c>
-      <c r="B29" s="0" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Todos los casos, incluidos los de smoke. Se ejecuta antes de cada entrega.</t>
         </is>
@@ -574,7 +590,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201, id=78, cvu=6882201591361058659598, alias=playa.aire.junco</t>
+          <t xml:space="preserve">HTTP 201, id=1, cvu=6334344006712411812213, alias=condor.relampago.laguna</t>
         </is>
       </c>
       <c r="P2" s="8" t="inlineStr">
@@ -656,7 +672,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cvu=0412676960179821491199 (22 dígitos)</t>
+          <t xml:space="preserve">cvu=4488830393826342522755 (22 dígitos)</t>
         </is>
       </c>
       <c r="P3" s="8" t="inlineStr">
@@ -738,7 +754,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">alias=viento.jardin.rocio (las 3 palabras están en alias-words.txt)</t>
+          <t xml:space="preserve">alias=arbol.tero.menta (las 3 palabras están en alias-words.txt)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -2296,7 +2312,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201 con id=91; login sin verificar: HTTP 403 (emailVerified ignorado)</t>
+          <t xml:space="preserve">HTTP 201 con id=14; login sin verificar: HTTP 403 (emailVerified ignorado)</t>
         </is>
       </c>
       <c r="P23" s="8" t="inlineStr">
@@ -2706,7 +2722,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sub=94, roles=['ROLE_USER'], vence en 60 min</t>
+          <t xml:space="preserve">sub=17, roles=['ROLE_USER'], vence en 60 min</t>
         </is>
       </c>
       <c r="P28" s="8" t="inlineStr">
@@ -3198,7 +3214,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: Juan Pérez &lt;qa857n34@mail.com&gt;</t>
+          <t xml:space="preserve">HTTP 200: Juan Pérez &lt;qa584n34@mail.com&gt;</t>
         </is>
       </c>
       <c r="P34" s="8" t="inlineStr">
@@ -4510,7 +4526,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mail "Digital Money House - Verificá tu email" con código de 6 dígitos (388095)</t>
+          <t xml:space="preserve">mail "Digital Money House - Verificá tu email" con código de 6 dígitos (275743)</t>
         </is>
       </c>
       <c r="P50" s="8" t="inlineStr">
@@ -6068,7 +6084,7 @@
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Swagger UI HTTP 200; auth: 7 endpoints, users: 2 endpoints, accounts: 5 endpoints</t>
+          <t xml:space="preserve">Swagger UI HTTP 200; auth: 7 endpoints, users: 2 endpoints, accounts: 8 endpoints</t>
         </is>
       </c>
       <c r="P69" s="8" t="inlineStr">
@@ -6478,7 +6494,7 @@
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: cvu=5121505547552248565229, alias=condor.bosque.perla, balance=0.0</t>
+          <t xml:space="preserve">HTTP 200: cvu=9412470896288656923251, alias=pasto.remo.tero, balance=0.0</t>
         </is>
       </c>
       <c r="P74" s="8" t="inlineStr">
@@ -6736,7 +6752,7 @@
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-105</t>
+          <t xml:space="preserve">TC-104</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
@@ -6751,27 +6767,27 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consultar la cuenta sin token</t>
+          <t xml:space="preserve">Los últimos movimientos son 5, del más reciente al más antiguo</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">—</t>
+          <t xml:space="preserve">Cuenta con 7 ingresos de $1 a $7.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GET /accounts/1 sin header Authorization.</t>
+          <t xml:space="preserve">GET /accounts/{accountId}/transactions.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 401.</t>
+          <t xml:space="preserve">HTTP 200 con 5 movimientos: 7, 6, 5, 4 y 3.</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seguridad</t>
+          <t xml:space="preserve">Positivo</t>
         </is>
       </c>
       <c r="I78" s="8" t="inlineStr">
@@ -6786,12 +6802,12 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Sprint3ApiTest.losUltimosMovimientosSonSolo5</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AccountApiTest.sinToken</t>
+          <t xml:space="preserve">ActivityApiTest.ultimosCinco</t>
         </is>
       </c>
       <c r="M78" s="8" t="inlineStr">
@@ -6806,7 +6822,7 @@
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 401</t>
+          <t xml:space="preserve">HTTP 200: [7.0, 6.0, 5.0, 4.0, 3.0]</t>
         </is>
       </c>
       <c r="P78" s="8" t="inlineStr">
@@ -6818,7 +6834,7 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-110</t>
+          <t xml:space="preserve">TC-105</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
@@ -6828,32 +6844,32 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2 Mi perfil</t>
+          <t xml:space="preserve">S2 Dashboard</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El perfil muestra los datos personales, el CVU y el alias</t>
+          <t xml:space="preserve">Consultar la cuenta sin token</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario logueado.</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GET /users/{userId} y GET /accounts/{accountId}.</t>
+          <t xml:space="preserve">GET /accounts/1 sin header Authorization.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ambos HTTP 200: datos personales sin contraseña; CVU y alias de la cuenta.</t>
+          <t xml:space="preserve">HTTP 401.</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Positivo</t>
+          <t xml:space="preserve">Seguridad</t>
         </is>
       </c>
       <c r="I79" s="8" t="inlineStr">
@@ -6863,17 +6879,17 @@
       </c>
       <c r="J79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smoke + Regresión</t>
+          <t xml:space="preserve">Regresión</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserApiTest.elUsuarioPuedeConsultarSusPropiosDatos</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserProfileApiTest.verPerfil</t>
+          <t xml:space="preserve">AccountApiTest.sinToken</t>
         </is>
       </c>
       <c r="M79" s="8" t="inlineStr">
@@ -6888,7 +6904,7 @@
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">usuario Juan Pérez; cvu=3060993157590059194827, alias=sabana.hielo.mapa</t>
+          <t xml:space="preserve">HTTP 401</t>
         </is>
       </c>
       <c r="P79" s="8" t="inlineStr">
@@ -6900,7 +6916,7 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-111</t>
+          <t xml:space="preserve">TC-110</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
@@ -6915,7 +6931,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Editar nombre y teléfono</t>
+          <t xml:space="preserve">El perfil muestra los datos personales, el CVU y el alias</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -6925,12 +6941,12 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PATCH /users/{userId} con {"firstName": "Juan Manuel", "phone": "+5491155556666"}.</t>
+          <t xml:space="preserve">GET /users/{userId} y GET /accounts/{accountId}.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200 con los datos nuevos; el apellido y el email no cambian.</t>
+          <t xml:space="preserve">Ambos HTTP 200: datos personales sin contraseña; CVU y alias de la cuenta.</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
@@ -6950,12 +6966,12 @@
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserApiTest.elUsuarioPuedeEditarNombreApellidoYTelefono</t>
+          <t xml:space="preserve">UserApiTest.elUsuarioPuedeConsultarSusPropiosDatos</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserProfileApiTest.editarPerfil</t>
+          <t xml:space="preserve">UserProfileApiTest.verPerfil</t>
         </is>
       </c>
       <c r="M80" s="8" t="inlineStr">
@@ -6970,7 +6986,7 @@
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: Juan Manuel Pérez, +5491155556666</t>
+          <t xml:space="preserve">usuario Juan Pérez; cvu=7356793963469973822129, alias=fogata.avion.glaciar</t>
         </is>
       </c>
       <c r="P80" s="8" t="inlineStr">
@@ -6982,7 +6998,7 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-112</t>
+          <t xml:space="preserve">TC-111</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
@@ -6997,7 +7013,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Editar sin enviar ningún dato</t>
+          <t xml:space="preserve">Editar nombre y teléfono</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -7007,37 +7023,37 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PATCH /users/{userId} con {}.</t>
+          <t xml:space="preserve">PATCH /users/{userId} con {"firstName": "Juan Manuel", "phone": "+5491155556666"}.</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400 indicando que hay que enviar al menos un dato.</t>
+          <t xml:space="preserve">HTTP 200 con los datos nuevos; el apellido y el email no cambian.</t>
         </is>
       </c>
       <c r="H81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Negativo</t>
+          <t xml:space="preserve">Positivo</t>
         </is>
       </c>
       <c r="I81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Media</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="J81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regresión</t>
+          <t xml:space="preserve">Smoke + Regresión</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserApiTest.editarSinDatosOConDatosInvalidosDevuelve400</t>
+          <t xml:space="preserve">UserApiTest.elUsuarioPuedeEditarNombreApellidoYTelefono</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserProfileApiTest.editarSinDatos</t>
+          <t xml:space="preserve">UserProfileApiTest.editarPerfil</t>
         </is>
       </c>
       <c r="M81" s="8" t="inlineStr">
@@ -7052,7 +7068,7 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400: Indique al menos un dato para modificar: firstName, lastName o phone</t>
+          <t xml:space="preserve">HTTP 200: Juan Manuel Pérez, +5491155556666</t>
         </is>
       </c>
       <c r="P81" s="8" t="inlineStr">
@@ -7064,7 +7080,7 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-113</t>
+          <t xml:space="preserve">TC-112</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
@@ -7079,7 +7095,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Editar con datos inválidos</t>
+          <t xml:space="preserve">Editar sin enviar ningún dato</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -7089,12 +7105,12 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PATCH /users/{userId} con firstName de solo espacios y phone = "123".</t>
+          <t xml:space="preserve">PATCH /users/{userId} con {}.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400 con un detalle por cada campo inválido.</t>
+          <t xml:space="preserve">HTTP 400 indicando que hay que enviar al menos un dato.</t>
         </is>
       </c>
       <c r="H82" s="8" t="inlineStr">
@@ -7119,7 +7135,7 @@
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserProfileApiTest.editarDatosInvalidos</t>
+          <t xml:space="preserve">UserProfileApiTest.editarSinDatos</t>
         </is>
       </c>
       <c r="M82" s="8" t="inlineStr">
@@ -7134,7 +7150,7 @@
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400: firstName: El nombre debe tener al menos una letra y solo letras, espacios, apóstrofes y guiones; phone: El teléfono debe tener entre 8 y 15 dígitos</t>
+          <t xml:space="preserve">HTTP 400: Indique al menos un dato para modificar: firstName, lastName o phone</t>
         </is>
       </c>
       <c r="P82" s="8" t="inlineStr">
@@ -7146,7 +7162,7 @@
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-114</t>
+          <t xml:space="preserve">TC-113</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
@@ -7161,7 +7177,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El email y el DNI no se modifican</t>
+          <t xml:space="preserve">Editar con datos inválidos</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -7171,22 +7187,22 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PATCH /users/{userId} con lastName, email y dni nuevos.</t>
+          <t xml:space="preserve">PATCH /users/{userId} con firstName de solo espacios y phone = "123".</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: cambia el apellido; el email y el DNI quedan como estaban.</t>
+          <t xml:space="preserve">HTTP 400 con un detalle por cada campo inválido.</t>
         </is>
       </c>
       <c r="H83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seguridad</t>
+          <t xml:space="preserve">Negativo</t>
         </is>
       </c>
       <c r="I83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Media</t>
         </is>
       </c>
       <c r="J83" s="8" t="inlineStr">
@@ -7196,12 +7212,12 @@
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserApiTest.elEmailYElDniNoSeModificanAunqueVenganEnElJson</t>
+          <t xml:space="preserve">UserApiTest.editarSinDatosOConDatosInvalidosDevuelve400</t>
         </is>
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserProfileApiTest.emailYDniNoEditables</t>
+          <t xml:space="preserve">UserProfileApiTest.editarDatosInvalidos</t>
         </is>
       </c>
       <c r="M83" s="8" t="inlineStr">
@@ -7216,7 +7232,7 @@
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: apellido=Gómez, email y DNI sin cambios</t>
+          <t xml:space="preserve">HTTP 400: firstName: El nombre debe tener al menos una letra y solo letras, espacios, apóstrofes y guiones; phone: El teléfono debe tener entre 8 y 15 dígitos</t>
         </is>
       </c>
       <c r="P83" s="8" t="inlineStr">
@@ -7228,7 +7244,7 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-115</t>
+          <t xml:space="preserve">TC-114</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
@@ -7243,22 +7259,22 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se pueden editar los datos de otro usuario</t>
+          <t xml:space="preserve">El email y el DNI no se modifican</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dos usuarios logueados.</t>
+          <t xml:space="preserve">Usuario logueado.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Con el token de A, PATCH /users/{userId de B}.</t>
+          <t xml:space="preserve">PATCH /users/{userId} con lastName, email y dni nuevos.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 403.</t>
+          <t xml:space="preserve">HTTP 200: cambia el apellido; el email y el DNI quedan como estaban.</t>
         </is>
       </c>
       <c r="H84" s="8" t="inlineStr">
@@ -7278,12 +7294,12 @@
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserApiTest.unUsuarioNoPuedeEditarLosDatosDeOtro</t>
+          <t xml:space="preserve">UserApiTest.elEmailYElDniNoSeModificanAunqueVenganEnElJson</t>
         </is>
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserProfileApiTest.editarOtroUsuario</t>
+          <t xml:space="preserve">UserProfileApiTest.emailYDniNoEditables</t>
         </is>
       </c>
       <c r="M84" s="8" t="inlineStr">
@@ -7298,7 +7314,7 @@
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 403</t>
+          <t xml:space="preserve">HTTP 200: apellido=Gómez, email y DNI sin cambios</t>
         </is>
       </c>
       <c r="P84" s="8" t="inlineStr">
@@ -7310,7 +7326,7 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-116</t>
+          <t xml:space="preserve">TC-115</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
@@ -7325,27 +7341,27 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modificar el alias de la cuenta</t>
+          <t xml:space="preserve">No se pueden editar los datos de otro usuario</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario logueado.</t>
+          <t xml:space="preserve">Dos usuarios logueados.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PATCH /accounts/{accountId} con {"alias": "Nuevo.Alias.Qa"} y luego GET /accounts/{accountId}.</t>
+          <t xml:space="preserve">Con el token de A, PATCH /users/{userId de B}.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200; el alias queda guardado en minúsculas.</t>
+          <t xml:space="preserve">HTTP 403.</t>
         </is>
       </c>
       <c r="H85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Positivo</t>
+          <t xml:space="preserve">Seguridad</t>
         </is>
       </c>
       <c r="I85" s="8" t="inlineStr">
@@ -7355,17 +7371,17 @@
       </c>
       <c r="J85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smoke + Regresión</t>
+          <t xml:space="preserve">Regresión</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.elDuenioPuedeCambiarSuAliasYSeGuardaEnMinusculas</t>
+          <t xml:space="preserve">UserApiTest.unUsuarioNoPuedeEditarLosDatosDeOtro</t>
         </is>
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AccountApiTest.modificarAlias</t>
+          <t xml:space="preserve">UserProfileApiTest.editarOtroUsuario</t>
         </is>
       </c>
       <c r="M85" s="8" t="inlineStr">
@@ -7380,7 +7396,7 @@
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: alias=nuevo.alias.qa132</t>
+          <t xml:space="preserve">HTTP 403</t>
         </is>
       </c>
       <c r="P85" s="8" t="inlineStr">
@@ -7392,7 +7408,7 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-117</t>
+          <t xml:space="preserve">TC-116</t>
         </is>
       </c>
       <c r="B86" s="8" t="inlineStr">
@@ -7407,7 +7423,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alias con formato inválido</t>
+          <t xml:space="preserve">Modificar el alias de la cuenta</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -7417,37 +7433,37 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PATCH /accounts/{accountId} con {"alias": "solo.dos"}.</t>
+          <t xml:space="preserve">PATCH /accounts/{accountId} con {"alias": "Nuevo.Alias.Qa"} y luego GET /accounts/{accountId}.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400.</t>
+          <t xml:space="preserve">HTTP 200; el alias queda guardado en minúsculas.</t>
         </is>
       </c>
       <c r="H86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Negativo</t>
+          <t xml:space="preserve">Positivo</t>
         </is>
       </c>
       <c r="I86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Media</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="J86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regresión</t>
+          <t xml:space="preserve">Smoke + Regresión</t>
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.unAliasConFormatoInvalidoDevuelve400</t>
+          <t xml:space="preserve">Sprint2ApiTest.elDuenioPuedeCambiarSuAliasYSeGuardaEnMinusculas</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AccountApiTest.aliasInvalido</t>
+          <t xml:space="preserve">AccountApiTest.modificarAlias</t>
         </is>
       </c>
       <c r="M86" s="8" t="inlineStr">
@@ -7462,7 +7478,7 @@
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400: alias: El alias debe tener tres palabras separadas por punto (letras y números)</t>
+          <t xml:space="preserve">HTTP 200: alias=nuevo.alias.qa56</t>
         </is>
       </c>
       <c r="P86" s="8" t="inlineStr">
@@ -7474,7 +7490,7 @@
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-118</t>
+          <t xml:space="preserve">TC-117</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
@@ -7489,22 +7505,22 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alias en uso por otra cuenta</t>
+          <t xml:space="preserve">Alias con formato inválido</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dos usuarios logueados.</t>
+          <t xml:space="preserve">Usuario logueado.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Con el token de B, PATCH /accounts/{accountId de B} con el alias de A.</t>
+          <t xml:space="preserve">PATCH /accounts/{accountId} con {"alias": "solo.dos"}.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 409.</t>
+          <t xml:space="preserve">HTTP 400.</t>
         </is>
       </c>
       <c r="H87" s="8" t="inlineStr">
@@ -7524,12 +7540,12 @@
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.unAliasYaUsadoPorOtraCuentaDevuelve409</t>
+          <t xml:space="preserve">Sprint2ApiTest.unAliasConFormatoInvalidoDevuelve400</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AccountApiTest.aliasEnUso</t>
+          <t xml:space="preserve">AccountApiTest.aliasInvalido</t>
         </is>
       </c>
       <c r="M87" s="8" t="inlineStr">
@@ -7544,7 +7560,7 @@
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 409: El alias camino.selva.globo ya está en uso</t>
+          <t xml:space="preserve">HTTP 400: alias: El alias debe tener tres palabras separadas por punto (letras y números)</t>
         </is>
       </c>
       <c r="P87" s="8" t="inlineStr">
@@ -7556,7 +7572,7 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-120</t>
+          <t xml:space="preserve">TC-118</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
@@ -7566,32 +7582,32 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2 Tarjetas</t>
+          <t xml:space="preserve">S2 Mi perfil</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin tarjetas la lista está vacía</t>
+          <t xml:space="preserve">Alias en uso por otra cuenta</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario logueado sin tarjetas.</t>
+          <t xml:space="preserve">Dos usuarios logueados.</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GET /accounts/{accountId}/cards.</t>
+          <t xml:space="preserve">Con el token de B, PATCH /accounts/{accountId de B} con el alias de A.</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200 con una lista vacía.</t>
+          <t xml:space="preserve">HTTP 409.</t>
         </is>
       </c>
       <c r="H88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Borde</t>
+          <t xml:space="preserve">Negativo</t>
         </is>
       </c>
       <c r="I88" s="8" t="inlineStr">
@@ -7606,12 +7622,12 @@
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.sinTarjetasLaListaEstaVacia</t>
+          <t xml:space="preserve">Sprint2ApiTest.unAliasYaUsadoPorOtraCuentaDevuelve409</t>
         </is>
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.listaVacia</t>
+          <t xml:space="preserve">AccountApiTest.aliasEnUso</t>
         </is>
       </c>
       <c r="M88" s="8" t="inlineStr">
@@ -7626,7 +7642,7 @@
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: []</t>
+          <t xml:space="preserve">HTTP 409: El alias rocio.panal.salto ya está en uso</t>
         </is>
       </c>
       <c r="P88" s="8" t="inlineStr">
@@ -7638,7 +7654,7 @@
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-121</t>
+          <t xml:space="preserve">TC-120</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
@@ -7653,47 +7669,47 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asociar una tarjeta a la cuenta</t>
+          <t xml:space="preserve">Sin tarjetas la lista está vacía</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario logueado.</t>
+          <t xml:space="preserve">Usuario logueado sin tarjetas.</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POST /accounts/{accountId}/cards con número válido, titular, vencimiento MM/AA, código y tipo.</t>
+          <t xml:space="preserve">GET /accounts/{accountId}/cards.</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201 con id, últimos 4 dígitos, marca, tipo y número enmascarado.</t>
+          <t xml:space="preserve">HTTP 200 con una lista vacía.</t>
         </is>
       </c>
       <c r="H89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Positivo</t>
+          <t xml:space="preserve">Borde</t>
         </is>
       </c>
       <c r="I89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Media</t>
         </is>
       </c>
       <c r="J89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smoke + Regresión</t>
+          <t xml:space="preserve">Regresión</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.asociarUnaTarjetaDevuelve201SinElNumeroCompletoNiElCodigo</t>
+          <t xml:space="preserve">Sprint2ApiTest.sinTarjetasLaListaEstaVacia</t>
         </is>
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.asociarTarjeta</t>
+          <t xml:space="preserve">CardApiTest.listaVacia</t>
         </is>
       </c>
       <c r="M89" s="8" t="inlineStr">
@@ -7708,7 +7724,7 @@
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201: VISA **** **** **** 7215, tipo DEBIT</t>
+          <t xml:space="preserve">HTTP 200: []</t>
         </is>
       </c>
       <c r="P89" s="8" t="inlineStr">
@@ -7720,7 +7736,7 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-122</t>
+          <t xml:space="preserve">TC-121</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
@@ -7735,22 +7751,22 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Listar las tarjetas de la cuenta</t>
+          <t xml:space="preserve">Asociar una tarjeta a la cuenta</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario con 2 tarjetas asociadas.</t>
+          <t xml:space="preserve">Usuario logueado.</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GET /accounts/{accountId}/cards.</t>
+          <t xml:space="preserve">POST /accounts/{accountId}/cards con número válido, titular, vencimiento MM/AA, código y tipo.</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200 con las 2 tarjetas.</t>
+          <t xml:space="preserve">HTTP 201 con id, últimos 4 dígitos, marca, tipo y número enmascarado.</t>
         </is>
       </c>
       <c r="H90" s="8" t="inlineStr">
@@ -7770,12 +7786,12 @@
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Sprint2ApiTest.asociarUnaTarjetaDevuelve201SinElNumeroCompletoNiElCodigo</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.listarTarjetas</t>
+          <t xml:space="preserve">CardApiTest.asociarTarjeta</t>
         </is>
       </c>
       <c r="M90" s="8" t="inlineStr">
@@ -7790,7 +7806,7 @@
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200 con 2 tarjetas</t>
+          <t xml:space="preserve">HTTP 201: VISA **** **** **** 0085, tipo DEBIT</t>
         </is>
       </c>
       <c r="P90" s="8" t="inlineStr">
@@ -7802,7 +7818,7 @@
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-123</t>
+          <t xml:space="preserve">TC-122</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
@@ -7817,22 +7833,22 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detalle de una tarjeta</t>
+          <t xml:space="preserve">Listar las tarjetas de la cuenta</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario con una tarjeta asociada.</t>
+          <t xml:space="preserve">Usuario con 2 tarjetas asociadas.</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GET /accounts/{accountId}/cards/{cardId}.</t>
+          <t xml:space="preserve">GET /accounts/{accountId}/cards.</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200 con los datos de la tarjeta.</t>
+          <t xml:space="preserve">HTTP 200 con las 2 tarjetas.</t>
         </is>
       </c>
       <c r="H91" s="8" t="inlineStr">
@@ -7842,22 +7858,22 @@
       </c>
       <c r="I91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Media</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="J91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regresión</t>
+          <t xml:space="preserve">Smoke + Regresión</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.detalleYEliminacionDeUnaTarjeta</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.detalleTarjeta</t>
+          <t xml:space="preserve">CardApiTest.listarTarjetas</t>
         </is>
       </c>
       <c r="M91" s="8" t="inlineStr">
@@ -7872,7 +7888,7 @@
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: tarjeta 13 terminada en 3198</t>
+          <t xml:space="preserve">HTTP 200 con 2 tarjetas</t>
         </is>
       </c>
       <c r="P91" s="8" t="inlineStr">
@@ -7884,7 +7900,7 @@
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-124</t>
+          <t xml:space="preserve">TC-123</t>
         </is>
       </c>
       <c r="B92" s="8" t="inlineStr">
@@ -7899,32 +7915,32 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una tarjeta asociada a otra cuenta no se puede volver a asociar</t>
+          <t xml:space="preserve">Detalle de una tarjeta</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarjeta asociada a la cuenta de A.</t>
+          <t xml:space="preserve">Usuario con una tarjeta asociada.</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Con el token de B, POST /accounts/{accountId de B}/cards con el mismo número.</t>
+          <t xml:space="preserve">GET /accounts/{accountId}/cards/{cardId}.</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 409 "La tarjeta ya está asociada a otra cuenta".</t>
+          <t xml:space="preserve">HTTP 200 con los datos de la tarjeta.</t>
         </is>
       </c>
       <c r="H92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Negativo</t>
+          <t xml:space="preserve">Positivo</t>
         </is>
       </c>
       <c r="I92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Media</t>
         </is>
       </c>
       <c r="J92" s="8" t="inlineStr">
@@ -7934,12 +7950,12 @@
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.unaTarjetaYaAsociadaAOtraCuentaDevuelve409</t>
+          <t xml:space="preserve">Sprint2ApiTest.detalleYEliminacionDeUnaTarjeta</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.tarjetaDeOtraCuenta</t>
+          <t xml:space="preserve">CardApiTest.detalleTarjeta</t>
         </is>
       </c>
       <c r="M92" s="8" t="inlineStr">
@@ -7954,7 +7970,7 @@
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 409: La tarjeta ya está asociada a otra cuenta</t>
+          <t xml:space="preserve">HTTP 200: tarjeta 5 terminada en 9557</t>
         </is>
       </c>
       <c r="P92" s="8" t="inlineStr">
@@ -7966,7 +7982,7 @@
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-125</t>
+          <t xml:space="preserve">TC-124</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
@@ -7981,22 +7997,22 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La misma tarjeta no se asocia dos veces a la misma cuenta</t>
+          <t xml:space="preserve">Una tarjeta asociada a otra cuenta no se puede volver a asociar</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarjeta ya asociada.</t>
+          <t xml:space="preserve">Tarjeta asociada a la cuenta de A.</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Repetir POST /accounts/{accountId}/cards con el mismo número.</t>
+          <t xml:space="preserve">Con el token de B, POST /accounts/{accountId de B}/cards con el mismo número.</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 409.</t>
+          <t xml:space="preserve">HTTP 409 "La tarjeta ya está asociada a otra cuenta".</t>
         </is>
       </c>
       <c r="H93" s="8" t="inlineStr">
@@ -8006,7 +8022,7 @@
       </c>
       <c r="I93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Media</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="J93" s="8" t="inlineStr">
@@ -8016,12 +8032,12 @@
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Sprint2ApiTest.unaTarjetaYaAsociadaAOtraCuentaDevuelve409</t>
         </is>
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.tarjetaRepetida</t>
+          <t xml:space="preserve">CardApiTest.tarjetaDeOtraCuenta</t>
         </is>
       </c>
       <c r="M93" s="8" t="inlineStr">
@@ -8036,7 +8052,7 @@
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 409: La tarjeta ya está asociada a esta cuenta</t>
+          <t xml:space="preserve">HTTP 409: La tarjeta ya está asociada a otra cuenta</t>
         </is>
       </c>
       <c r="P93" s="8" t="inlineStr">
@@ -8048,7 +8064,7 @@
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-126</t>
+          <t xml:space="preserve">TC-125</t>
         </is>
       </c>
       <c r="B94" s="8" t="inlineStr">
@@ -8063,22 +8079,22 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Número de tarjeta inválido (dígito verificador)</t>
+          <t xml:space="preserve">La misma tarjeta no se asocia dos veces a la misma cuenta</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario logueado.</t>
+          <t xml:space="preserve">Tarjeta ya asociada.</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POST /accounts/{accountId}/cards con el número 4509953566233705.</t>
+          <t xml:space="preserve">Repetir POST /accounts/{accountId}/cards con el mismo número.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400 "El número de tarjeta no es válido".</t>
+          <t xml:space="preserve">HTTP 409.</t>
         </is>
       </c>
       <c r="H94" s="8" t="inlineStr">
@@ -8098,12 +8114,12 @@
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.unNumeroQueNoPasaLuhnDevuelve400</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.numeroInvalido</t>
+          <t xml:space="preserve">CardApiTest.tarjetaRepetida</t>
         </is>
       </c>
       <c r="M94" s="8" t="inlineStr">
@@ -8118,7 +8134,7 @@
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400: El número de tarjeta no es válido</t>
+          <t xml:space="preserve">HTTP 409: La tarjeta ya está asociada a esta cuenta</t>
         </is>
       </c>
       <c r="P94" s="8" t="inlineStr">
@@ -8130,7 +8146,7 @@
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-127</t>
+          <t xml:space="preserve">TC-126</t>
         </is>
       </c>
       <c r="B95" s="8" t="inlineStr">
@@ -8145,7 +8161,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarjeta vencida</t>
+          <t xml:space="preserve">Número de tarjeta inválido (dígito verificador)</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -8155,12 +8171,12 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POST /accounts/{accountId}/cards con vencimiento 01/20.</t>
+          <t xml:space="preserve">POST /accounts/{accountId}/cards con el número 4509953566233705.</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400 "La tarjeta está vencida".</t>
+          <t xml:space="preserve">HTTP 400 "El número de tarjeta no es válido".</t>
         </is>
       </c>
       <c r="H95" s="8" t="inlineStr">
@@ -8180,12 +8196,12 @@
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.unaTarjetaVencidaDevuelve400</t>
+          <t xml:space="preserve">Sprint2ApiTest.unNumeroQueNoPasaLuhnDevuelve400</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.tarjetaVencida</t>
+          <t xml:space="preserve">CardApiTest.numeroInvalido</t>
         </is>
       </c>
       <c r="M95" s="8" t="inlineStr">
@@ -8200,7 +8216,7 @@
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400: La tarjeta está vencida</t>
+          <t xml:space="preserve">HTTP 400: El número de tarjeta no es válido</t>
         </is>
       </c>
       <c r="P95" s="8" t="inlineStr">
@@ -8212,7 +8228,7 @@
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-128</t>
+          <t xml:space="preserve">TC-127</t>
         </is>
       </c>
       <c r="B96" s="8" t="inlineStr">
@@ -8227,7 +8243,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Datos de tarjeta faltantes</t>
+          <t xml:space="preserve">Tarjeta vencida</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -8237,12 +8253,12 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POST /accounts/{accountId}/cards con {}.</t>
+          <t xml:space="preserve">POST /accounts/{accountId}/cards con vencimiento 01/20.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400 con un detalle por cada uno de los 5 campos.</t>
+          <t xml:space="preserve">HTTP 400 "La tarjeta está vencida".</t>
         </is>
       </c>
       <c r="H96" s="8" t="inlineStr">
@@ -8262,12 +8278,12 @@
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.datosDeTarjetaFaltantesDevuelven400ConElDetalle</t>
+          <t xml:space="preserve">Sprint2ApiTest.unaTarjetaVencidaDevuelve400</t>
         </is>
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.datosFaltantes</t>
+          <t xml:space="preserve">CardApiTest.tarjetaVencida</t>
         </is>
       </c>
       <c r="M96" s="8" t="inlineStr">
@@ -8282,7 +8298,7 @@
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 400 con 5 detalles</t>
+          <t xml:space="preserve">HTTP 400: La tarjeta está vencida</t>
         </is>
       </c>
       <c r="P96" s="8" t="inlineStr">
@@ -8294,7 +8310,7 @@
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-129</t>
+          <t xml:space="preserve">TC-128</t>
         </is>
       </c>
       <c r="B97" s="8" t="inlineStr">
@@ -8309,47 +8325,47 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eliminar una tarjeta</t>
+          <t xml:space="preserve">Datos de tarjeta faltantes</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario con una tarjeta asociada.</t>
+          <t xml:space="preserve">Usuario logueado.</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DELETE /accounts/{accountId}/cards/{cardId} y luego listar las tarjetas.</t>
+          <t xml:space="preserve">POST /accounts/{accountId}/cards con {}.</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200; la tarjeta ya no aparece en la lista.</t>
+          <t xml:space="preserve">HTTP 400 con un detalle por cada uno de los 5 campos.</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Positivo</t>
+          <t xml:space="preserve">Negativo</t>
         </is>
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Media</t>
         </is>
       </c>
       <c r="J97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smoke + Regresión</t>
+          <t xml:space="preserve">Regresión</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.detalleYEliminacionDeUnaTarjeta</t>
+          <t xml:space="preserve">Sprint2ApiTest.datosDeTarjetaFaltantesDevuelven400ConElDetalle</t>
         </is>
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.eliminarTarjeta</t>
+          <t xml:space="preserve">CardApiTest.datosFaltantes</t>
         </is>
       </c>
       <c r="M97" s="8" t="inlineStr">
@@ -8364,7 +8380,7 @@
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200; la lista quedó vacía</t>
+          <t xml:space="preserve">HTTP 400 con 5 detalles</t>
         </is>
       </c>
       <c r="P97" s="8" t="inlineStr">
@@ -8376,7 +8392,7 @@
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-130</t>
+          <t xml:space="preserve">TC-129</t>
         </is>
       </c>
       <c r="B98" s="8" t="inlineStr">
@@ -8391,37 +8407,37 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eliminar una tarjeta inexistente</t>
+          <t xml:space="preserve">Eliminar una tarjeta</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario logueado.</t>
+          <t xml:space="preserve">Usuario con una tarjeta asociada.</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DELETE /accounts/{accountId}/cards/999999.</t>
+          <t xml:space="preserve">DELETE /accounts/{accountId}/cards/{cardId} y luego listar las tarjetas.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404.</t>
+          <t xml:space="preserve">HTTP 200; la tarjeta ya no aparece en la lista.</t>
         </is>
       </c>
       <c r="H98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Negativo</t>
+          <t xml:space="preserve">Positivo</t>
         </is>
       </c>
       <c r="I98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Media</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="J98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regresión</t>
+          <t xml:space="preserve">Smoke + Regresión</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
@@ -8431,7 +8447,7 @@
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.eliminarInexistente</t>
+          <t xml:space="preserve">CardApiTest.eliminarTarjeta</t>
         </is>
       </c>
       <c r="M98" s="8" t="inlineStr">
@@ -8446,7 +8462,7 @@
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404: No existe la tarjeta 999999 asociada a la cuenta 147</t>
+          <t xml:space="preserve">HTTP 200; la lista quedó vacía</t>
         </is>
       </c>
       <c r="P98" s="8" t="inlineStr">
@@ -8458,7 +8474,7 @@
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-131</t>
+          <t xml:space="preserve">TC-130</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
@@ -8473,32 +8489,32 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Las tarjetas de otra cuenta no son accesibles</t>
+          <t xml:space="preserve">Eliminar una tarjeta inexistente</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A tiene una tarjeta; B logueado.</t>
+          <t xml:space="preserve">Usuario logueado.</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Con el token de B: listar las tarjetas de A, y ver y eliminar la tarjeta de A usando la cuenta de B.</t>
+          <t xml:space="preserve">DELETE /accounts/{accountId}/cards/999999.</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Listado ajeno: HTTP 403. Ver y eliminar desde otra cuenta: HTTP 404. La tarjeta de A sigue existiendo.</t>
+          <t xml:space="preserve">HTTP 404.</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seguridad</t>
+          <t xml:space="preserve">Negativo</t>
         </is>
       </c>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Media</t>
         </is>
       </c>
       <c r="J99" s="8" t="inlineStr">
@@ -8508,12 +8524,12 @@
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint2ApiTest.unaTarjetaDeOtraCuentaNoSePuedeVerNiEliminarDesdeLaPropia</t>
+          <t xml:space="preserve">Sprint2ApiTest.detalleYEliminacionDeUnaTarjeta</t>
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardApiTest.tarjetasAjenas</t>
+          <t xml:space="preserve">CardApiTest.eliminarInexistente</t>
         </is>
       </c>
       <c r="M99" s="8" t="inlineStr">
@@ -8528,7 +8544,7 @@
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">listado ajeno 403; ver y borrar desde otra cuenta 404; la tarjeta de A sigue</t>
+          <t xml:space="preserve">HTTP 404: No existe la tarjeta 999999 asociada a la cuenta 71</t>
         </is>
       </c>
       <c r="P99" s="8" t="inlineStr">
@@ -8540,87 +8556,1891 @@
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">TC-131</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2 Tarjetas</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Las tarjetas de otra cuenta no son accesibles</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A tiene una tarjeta; B logueado.</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con el token de B: listar las tarjetas de A, y ver y eliminar la tarjeta de A usando la cuenta de B.</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Listado ajeno: HTTP 403. Ver y eliminar desde otra cuenta: HTTP 404. La tarjeta de A sigue existiendo.</t>
+        </is>
+      </c>
+      <c r="H100" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J100" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint2ApiTest.unaTarjetaDeOtraCuentaNoSePuedeVerNiEliminarDesdeLaPropia</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CardApiTest.tarjetasAjenas</t>
+        </is>
+      </c>
+      <c r="M100" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N100" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">listado ajeno 403; ver y borrar desde otra cuenta 404; la tarjeta de A sigue</t>
+        </is>
+      </c>
+      <c r="P100" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">TC-132</t>
         </is>
       </c>
-      <c r="B100" s="8" t="inlineStr">
+      <c r="B101" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
+      <c r="C101" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">S2 Tarjetas</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="D101" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">La API no expone el número completo ni el código de seguridad</t>
         </is>
       </c>
-      <c r="E100" s="2" t="inlineStr">
+      <c r="E101" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Usuario logueado.</t>
         </is>
       </c>
-      <c r="F100" s="2" t="inlineStr">
+      <c r="F101" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Asociar una tarjeta y revisar la respuesta y el listado.</t>
         </is>
       </c>
-      <c r="G100" s="2" t="inlineStr">
+      <c r="G101" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ninguna respuesta contiene el número completo ni un campo cvv.</t>
         </is>
       </c>
-      <c r="H100" s="8" t="inlineStr">
+      <c r="H101" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Seguridad</t>
         </is>
       </c>
-      <c r="I100" s="8" t="inlineStr">
+      <c r="I101" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Alta</t>
         </is>
       </c>
-      <c r="J100" s="8" t="inlineStr">
+      <c r="J101" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Regresión</t>
         </is>
       </c>
-      <c r="K100" s="2" t="inlineStr">
+      <c r="K101" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="L100" s="2" t="inlineStr">
+      <c r="L101" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">CardApiTest.noExponeDatosSensibles</t>
         </is>
       </c>
-      <c r="M100" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Script</t>
-        </is>
-      </c>
-      <c r="N100" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pasó</t>
-        </is>
-      </c>
-      <c r="O100" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">solo se expone **** **** **** 8400</t>
-        </is>
-      </c>
-      <c r="P100" s="8" t="inlineStr">
+      <c r="M101" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N101" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">solo se expone **** **** **** 7084</t>
+        </is>
+      </c>
+      <c r="P101" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-140</t>
+        </is>
+      </c>
+      <c r="B102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Toda la actividad, de la más reciente a la más antigua</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta con 3 ingresos.</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity con el token del dueño.</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con los 3 movimientos, el más reciente primero.</t>
+        </is>
+      </c>
+      <c r="H102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.laActividadListaTodoDelMasRecienteAlMasAntiguo</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.actividadOrdenada</t>
+        </is>
+      </c>
+      <c r="M102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N102" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200: ids [10, 9, 8]</t>
+        </is>
+      </c>
+      <c r="P102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-141</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actividad de una cuenta sin movimientos</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta nueva.</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity.</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con una lista vacía.</t>
+        </is>
+      </c>
+      <c r="H103" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borde</t>
+        </is>
+      </c>
+      <c r="I103" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J103" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.actividadVacia</t>
+        </is>
+      </c>
+      <c r="M103" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N103" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200: []</t>
+        </is>
+      </c>
+      <c r="P103" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-142</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actividad de otra cuenta</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dos usuarios logueados.</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con el token de A, GET /accounts/{accountId de B}/activity.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 403.</t>
+        </is>
+      </c>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J104" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.laActividadDeOtraCuentaDevuelve403</t>
+        </is>
+      </c>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.actividadAjena</t>
+        </is>
+      </c>
+      <c r="M104" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N104" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 403</t>
+        </is>
+      </c>
+      <c r="P104" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-143</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actividad sin token</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/1/activity sin header Authorization.</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 401.</t>
+        </is>
+      </c>
+      <c r="H105" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I105" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J105" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.actividadSinToken</t>
+        </is>
+      </c>
+      <c r="M105" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N105" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O105" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 401</t>
+        </is>
+      </c>
+      <c r="P105" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-144</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle de una actividad</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta con un ingreso de $250.</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity/{id del movimiento}.</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con tipo, monto, fecha, descripción y tarjeta.</t>
+        </is>
+      </c>
+      <c r="H106" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J106" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.detalleDeUnaActividad</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.detalle</t>
+        </is>
+      </c>
+      <c r="M106" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N106" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200: DEPOSIT $250.0 - Ingreso desde tarjeta terminada en 3971</t>
+        </is>
+      </c>
+      <c r="P106" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-145</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle de una actividad inexistente</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario logueado.</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity/999999.</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 404.</t>
+        </is>
+      </c>
+      <c r="H107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.detalleInexistenteOdeOtraCuentaDevuelve404</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.detalleInexistente</t>
+        </is>
+      </c>
+      <c r="M107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N107" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 404: No existe la actividad 999999 en la cuenta 80</t>
+        </is>
+      </c>
+      <c r="P107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-146</t>
+        </is>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle de un movimiento de otra cuenta</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A tiene un movimiento; B logueado.</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con el token de B: pedir el movimiento de A usando la cuenta de B, y usando la cuenta de A.</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Desde la cuenta de B: HTTP 404. Usando la cuenta de A: HTTP 403.</t>
+        </is>
+      </c>
+      <c r="H108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.detalleInexistenteOdeOtraCuentaDevuelve404</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.detalleAjeno</t>
+        </is>
+      </c>
+      <c r="M108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N108" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">desde la cuenta propia 404; usando la cuenta ajena 403</t>
+        </is>
+      </c>
+      <c r="P108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-147</t>
+        </is>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle con id inválido</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario logueado.</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity/abc.</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400.</t>
+        </is>
+      </c>
+      <c r="H109" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I109" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja</t>
+        </is>
+      </c>
+      <c r="J109" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.detalleIdInvalido</t>
+        </is>
+      </c>
+      <c r="M109" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N109" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400</t>
+        </is>
+      </c>
+      <c r="P109" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-150</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingresar dinero desde una tarjeta propia</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario con una tarjeta asociada y saldo 0.</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POST /accounts/{accountId}/transferences con {"cardId": id, "amount": 1500.50}. Luego GET /accounts/{accountId}.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 201 con el movimiento (DEPOSIT, INCOME, 1500.50). El saldo pasa a 1500.50.</t>
+        </is>
+      </c>
+      <c r="H110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.ingresarDineroDesdeUnaTarjetaDevuelve201YSumaAlSaldo</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.ingresarDinero</t>
+        </is>
+      </c>
+      <c r="M110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N110" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 201; saldo 1500.5</t>
+        </is>
+      </c>
+      <c r="P110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-151</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingresar con una tarjeta de otra cuenta</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A tiene una tarjeta; B logueado.</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con el token de B, POST /accounts/{accountId de B}/transferences con la tarjeta de A.</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 404 y el saldo de B no cambia.</t>
+        </is>
+      </c>
+      <c r="H111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.ingresarConUnaTarjetaDeOtraCuentaDevuelve404YNoCambiaElSaldo</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.tarjetaDeOtraCuenta</t>
+        </is>
+      </c>
+      <c r="M111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N111" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O111" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 404; saldo de B sin cambios</t>
+        </is>
+      </c>
+      <c r="P111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-152</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montos inválidos</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario con una tarjeta.</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingresar 0, -10, 10.555 y 1000000.01.</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 en los cuatro casos; el saldo no cambia.</t>
+        </is>
+      </c>
+      <c r="H112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.montosInvalidosDevuelven400</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.montosInvalidos</t>
+        </is>
+      </c>
+      <c r="M112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N112" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 en los 4 montos; saldo 0</t>
+        </is>
+      </c>
+      <c r="P112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-153</t>
+        </is>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monto o tarjeta enviados como texto</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario con una tarjeta.</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingresar con "amount": "100" y con "cardId": "&lt;id&gt;" (entre comillas).</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 en ambos.</t>
+        </is>
+      </c>
+      <c r="H113" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I113" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J113" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.montoYTarjetaEnviadosComoTextoDevuelven400</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.tiposIncorrectos</t>
+        </is>
+      </c>
+      <c r="M113" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N113" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O113" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 en ambos</t>
+        </is>
+      </c>
+      <c r="P113" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-154</t>
+        </is>
+      </c>
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingreso sin indicar la tarjeta</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario logueado.</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POST /accounts/{accountId}/transferences con {"amount": 100}.</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400.</t>
+        </is>
+      </c>
+      <c r="H114" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I114" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J114" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.sinTarjetaNiDestinoOConAmbosDevuelve400</t>
+        </is>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.sinTarjeta</t>
+        </is>
+      </c>
+      <c r="M114" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N114" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400: oneOperation: Indique cardId (ingreso desde tarjeta) o destination (transferencia), pero no ambos</t>
+        </is>
+      </c>
+      <c r="P114" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-155</t>
+        </is>
+      </c>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No se puede ingresar dinero en una cuenta ajena</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A tiene una tarjeta; B logueado.</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con el token de B, POST /accounts/{accountId de A}/transferences.</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 403.</t>
+        </is>
+      </c>
+      <c r="H115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.noSePuedeIngresarDineroEnUnaCuentaAjena</t>
+        </is>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.cuentaAjena</t>
+        </is>
+      </c>
+      <c r="M115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N115" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O115" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 403</t>
+        </is>
+      </c>
+      <c r="P115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-156</t>
+        </is>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El ingreso aparece en la actividad y en los últimos movimientos</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario con una tarjeta.</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingresar $250 y consultar /activity y /transactions.</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El movimiento es el primero de ambas listas.</t>
+        </is>
+      </c>
+      <c r="H116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.ingresoVisibleEnActividad</t>
+        </is>
+      </c>
+      <c r="M116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N116" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">primero en /activity y en /transactions</t>
+        </is>
+      </c>
+      <c r="P116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-157</t>
+        </is>
+      </c>
+      <c r="B117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Una tarjeta eliminada no se puede usar y sus ingresos conservan los datos</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario con un ingreso hecho con una tarjeta.</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eliminar la tarjeta, intentar otro ingreso con ella y consultar el detalle del ingreso anterior.</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nuevo ingreso: HTTP 404. El detalle anterior sigue mostrando los últimos 4 dígitos de la tarjeta.</t>
+        </is>
+      </c>
+      <c r="H117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borde</t>
+        </is>
+      </c>
+      <c r="I117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N117" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nuevo ingreso 404; el detalle conserva la tarjeta ...6404</t>
+        </is>
+      </c>
+      <c r="P117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-158</t>
+        </is>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingresos simultáneos no pierden dinero</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario con una tarjeta.</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enviar 10 ingresos de $100 al mismo tiempo (10 hilos).</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los 10 responden 201 y el saldo final es $1000.</t>
+        </is>
+      </c>
+      <c r="H118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borde</t>
+        </is>
+      </c>
+      <c r="I118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.ingresosSimultaneosNoPierdenDinero</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N118" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10 respuestas 201; saldo 1000.0</t>
+        </is>
+      </c>
+      <c r="P118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-160</t>
+        </is>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Opcional: filtros</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtrar la actividad por rango de monto</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta con ingresos de $500, $3.000 y $150.000.</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity?minAmount=1000&amp;maxAmount=5000 y ?minAmount=100000.</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Primer filtro: solo $3.000. Segundo: solo $150.000.</t>
+        </is>
+      </c>
+      <c r="H119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.filtrosPorMontoTipoYFecha</t>
+        </is>
+      </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.filtroPorMonto</t>
+        </is>
+      </c>
+      <c r="M119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N119" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$1.000-$5.000: [3000.0]; más de $100.000: [150000.0]</t>
+        </is>
+      </c>
+      <c r="P119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-161</t>
+        </is>
+      </c>
+      <c r="B120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Opcional: filtros</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtrar la actividad por ingreso o egreso</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta con un ingreso.</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity?direction=income y ?direction=EXPENSE.</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INCOME (sin importar mayúsculas): 1 movimiento. EXPENSE: lista vacía.</t>
+        </is>
+      </c>
+      <c r="H120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.elFiltroDeTipoNoDistingueMayusculasYLosErroresNoExponenClasesInternas</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.filtroPorTipo</t>
+        </is>
+      </c>
+      <c r="M120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N120" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ingresos: 1; egresos: 0</t>
+        </is>
+      </c>
+      <c r="P120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-162</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Opcional: filtros</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtrar la actividad por período</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta con un ingreso de hoy.</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity?from=2000-01-01&amp;to=2000-12-31 y ?from=2000-01-01.</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Primer período: lista vacía. Segundo: el ingreso.</t>
+        </is>
+      </c>
+      <c r="H121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.filtrosPorMontoTipoYFecha</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.filtroPorPeriodo</t>
+        </is>
+      </c>
+      <c r="M121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N121" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O121" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">año 2000: 0 movimientos; desde 2000: 1</t>
+        </is>
+      </c>
+      <c r="P121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-163</t>
+        </is>
+      </c>
+      <c r="B122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Opcional: filtros</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtros inválidos</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario logueado.</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">from posterior a to; minAmount mayor que maxAmount; minAmount=abc.</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 en los tres casos, sin nombres de clases internas en el mensaje.</t>
+        </is>
+      </c>
+      <c r="H122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.filtrosInvalidosDevuelven400</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.filtrosInvalidos</t>
+        </is>
+      </c>
+      <c r="M122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N122" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O122" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 en los tres; minAmount: tiene un valor inválido</t>
+        </is>
+      </c>
+      <c r="P122" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">15/10/2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P100"/>
+  <autoFilter ref="A1:P122"/>
 </worksheet>
 </file>
 
@@ -8800,7 +10620,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201, id=78, cvu=6882201591361058659598, alias=playa.aire.junco</t>
+          <t xml:space="preserve">HTTP 201, id=1, cvu=6334344006712411812213, alias=condor.relampago.laguna</t>
         </is>
       </c>
       <c r="P2" s="8" t="inlineStr">
@@ -8964,7 +10784,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: Juan Pérez &lt;qa857n34@mail.com&gt;</t>
+          <t xml:space="preserve">HTTP 200: Juan Pérez &lt;qa584n34@mail.com&gt;</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -9538,7 +11358,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: cvu=5121505547552248565229, alias=condor.bosque.perla, balance=0.0</t>
+          <t xml:space="preserve">HTTP 200: cvu=9412470896288656923251, alias=pasto.remo.tero, balance=0.0</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
@@ -9620,7 +11440,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">usuario Juan Pérez; cvu=3060993157590059194827, alias=sabana.hielo.mapa</t>
+          <t xml:space="preserve">usuario Juan Pérez; cvu=7356793963469973822129, alias=fogata.avion.glaciar</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
@@ -9784,7 +11604,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: alias=nuevo.alias.qa132</t>
+          <t xml:space="preserve">HTTP 200: alias=nuevo.alias.qa56</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
@@ -9866,7 +11686,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201: VISA **** **** **** 7215, tipo DEBIT</t>
+          <t xml:space="preserve">HTTP 201: VISA **** **** **** 0085, tipo DEBIT</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
@@ -10039,7 +11859,253 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-140</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Toda la actividad, de la más reciente a la más antigua</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta con 3 ingresos.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity con el token del dueño.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con los 3 movimientos, el más reciente primero.</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.laActividadListaTodoDelMasRecienteAlMasAntiguo</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.actividadOrdenada</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200: ids [10, 9, 8]</t>
+        </is>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-144</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Mi actividad</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle de una actividad</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta con un ingreso de $250.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity/{id del movimiento}.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con tipo, monto, fecha, descripción y tarjeta.</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.detalleDeUnaActividad</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.detalle</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200: DEPOSIT $250.0 - Ingreso desde tarjeta terminada en 3971</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-150</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingresar dinero desde una tarjeta propia</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario con una tarjeta asociada y saldo 0.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POST /accounts/{accountId}/transferences con {"cardId": id, "amount": 1500.50}. Luego GET /accounts/{accountId}.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 201 con el movimiento (DEPOSIT, INCOME, 1500.50). El saldo pasa a 1500.50.</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint3ApiTest.ingresarDineroDesdeUnaTarjetaDevuelve201YSumaAlSaldo</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ActivityApiTest.ingresarDinero</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 201; saldo 1500.5</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P17"/>
+  <autoFilter ref="A1:P20"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: QA sign-off, exploratorio del sprint 4 e informe de los sprints 2 a 4
- TC-086 y TC-087 (entorno Docker con MySQL) pasan en GitHub Actions (CI #4):
  la planilla queda con 138 de 138 casos aprobados.
- QA sign-off con las metricas pedidas, testing exploratorio del sprint 4,
  guia de la coleccion de Postman e informe en HTML y PDF.
- README con los endpoints de los sprints 2 a 4 y la integracion continua.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/casos-de-prueba.xlsx
+++ b/docs/testing/casos-de-prueba.xlsx
@@ -140,7 +140,7 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-15 12:35:33</t>
+          <t xml:space="preserve">2026-10-15 12:59:21</t>
         </is>
       </c>
     </row>
@@ -340,7 +340,7 @@
         <v>72</v>
       </c>
       <c r="C24" s="8">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D24" s="8">
         <v>12</v>
@@ -378,33 +378,49 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Criterios</t>
-        </is>
-      </c>
-    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 4</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <v>17</v>
+      </c>
+      <c r="C27" s="8">
+        <v>17</v>
+      </c>
+      <c r="D27" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smoke</t>
-        </is>
-      </c>
-      <c r="B29" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Camino feliz de cada historia y verificaciones mínimas de seguridad e infraestructura. Si falla, el build no es apto para seguir probando.</t>
+          <t xml:space="preserve">Criterios</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Smoke</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Camino feliz de cada historia y verificaciones mínimas de seguridad e infraestructura. Si falla, el build no es apto para seguir probando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Regresión</t>
         </is>
       </c>
-      <c r="B30" s="0" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Todos los casos, incluidos los de smoke. Se ejecuta antes de cada entrega.</t>
         </is>
@@ -590,7 +606,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201, id=1, cvu=6334344006712411812213, alias=condor.relampago.laguna</t>
+          <t xml:space="preserve">HTTP 201, id=98, cvu=3257469782009407052174, alias=roca.delta.agua</t>
         </is>
       </c>
       <c r="P2" s="8" t="inlineStr">
@@ -672,7 +688,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cvu=4488830393826342522755 (22 dígitos)</t>
+          <t xml:space="preserve">cvu=2437004423526538058333 (22 dígitos)</t>
         </is>
       </c>
       <c r="P3" s="8" t="inlineStr">
@@ -754,7 +770,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">alias=arbol.tero.menta (las 3 palabras están en alias-words.txt)</t>
+          <t xml:space="preserve">alias=rocio.canoa.hongo (las 3 palabras están en alias-words.txt)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -2312,7 +2328,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201 con id=14; login sin verificar: HTTP 403 (emailVerified ignorado)</t>
+          <t xml:space="preserve">HTTP 201 con id=111; login sin verificar: HTTP 403 (emailVerified ignorado)</t>
         </is>
       </c>
       <c r="P23" s="8" t="inlineStr">
@@ -2722,7 +2738,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sub=17, roles=['ROLE_USER'], vence en 60 min</t>
+          <t xml:space="preserve">sub=114, roles=['ROLE_USER'], vence en 60 min</t>
         </is>
       </c>
       <c r="P28" s="8" t="inlineStr">
@@ -3214,7 +3230,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: Juan Pérez &lt;qa584n34@mail.com&gt;</t>
+          <t xml:space="preserve">HTTP 200: Juan Pérez &lt;qa439n34@mail.com&gt;</t>
         </is>
       </c>
       <c r="P34" s="8" t="inlineStr">
@@ -4526,7 +4542,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mail "Digital Money House - Verificá tu email" con código de 6 dígitos (275743)</t>
+          <t xml:space="preserve">mail "Digital Money House - Verificá tu email" con código de 6 dígitos (119713)</t>
         </is>
       </c>
       <c r="P50" s="8" t="inlineStr">
@@ -6084,7 +6100,7 @@
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Swagger UI HTTP 200; auth: 7 endpoints, users: 2 endpoints, accounts: 8 endpoints</t>
+          <t xml:space="preserve">Swagger UI HTTP 200; auth: 7 endpoints, users: 2 endpoints, accounts: 9 endpoints</t>
         </is>
       </c>
       <c r="P69" s="8" t="inlineStr">
@@ -6323,19 +6339,19 @@
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="N72" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bloqueado</t>
+      <c r="N72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se pudo ejecutar: en esta máquina Docker Desktop no arranca porque Windows no tiene habilitada la característica "Plataforma de máquina virtual" (requiere administrador y reinicio). docker compose config valida el archivo.</t>
+          <t xml:space="preserve">Ejecutado en GitHub Actions (job docker-e2e, CI #4, commit 08442ee): docker compose up -d --build levantó MySQL, MailHog y los 5 servicios; los 4 servicios quedaron UP en Eureka y la automatización RestAssured (75 de 75) y la suite de casos pasaron contra MySQL y MailHog.</t>
         </is>
       </c>
       <c r="P72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">02/10/2026</t>
+          <t xml:space="preserve">15/10/2026</t>
         </is>
       </c>
     </row>
@@ -6405,19 +6421,19 @@
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="N73" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bloqueado</t>
+      <c r="N73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
         </is>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Depende de TC-086 (Docker). La suite se ejecutó con el perfil h2 (base en memoria).</t>
+          <t xml:space="preserve">Ejecutado en GitHub Actions (job docker-e2e, CI #4, commit 08442ee) con scripts/check_persistence.py: después de docker compose restart de users-service, account-service y auth-service, el login respondió HTTP 200 y la cuenta conservó CVU, saldo 1234.50 y su movimiento.</t>
         </is>
       </c>
       <c r="P73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">02/10/2026</t>
+          <t xml:space="preserve">15/10/2026</t>
         </is>
       </c>
     </row>
@@ -6494,7 +6510,7 @@
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: cvu=9412470896288656923251, alias=pasto.remo.tero, balance=0.0</t>
+          <t xml:space="preserve">HTTP 200: cvu=9713684828224062434639, alias=pradera.perla.trueno, balance=0.0</t>
         </is>
       </c>
       <c r="P74" s="8" t="inlineStr">
@@ -6986,7 +7002,7 @@
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">usuario Juan Pérez; cvu=7356793963469973822129, alias=fogata.avion.glaciar</t>
+          <t xml:space="preserve">usuario Juan Pérez; cvu=6658065001634942495360, alias=tigre.yaguarete.remo</t>
         </is>
       </c>
       <c r="P80" s="8" t="inlineStr">
@@ -7478,7 +7494,7 @@
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: alias=nuevo.alias.qa56</t>
+          <t xml:space="preserve">HTTP 200: alias=nuevo.alias.qa153</t>
         </is>
       </c>
       <c r="P86" s="8" t="inlineStr">
@@ -7642,7 +7658,7 @@
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 409: El alias rocio.panal.salto ya está en uso</t>
+          <t xml:space="preserve">HTTP 409: El alias volcan.cima.rio ya está en uso</t>
         </is>
       </c>
       <c r="P88" s="8" t="inlineStr">
@@ -7806,7 +7822,7 @@
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201: VISA **** **** **** 0085, tipo DEBIT</t>
+          <t xml:space="preserve">HTTP 201: VISA **** **** **** 4931, tipo DEBIT</t>
         </is>
       </c>
       <c r="P90" s="8" t="inlineStr">
@@ -7970,7 +7986,7 @@
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: tarjeta 5 terminada en 9557</t>
+          <t xml:space="preserve">HTTP 200: tarjeta 43 terminada en 9261</t>
         </is>
       </c>
       <c r="P92" s="8" t="inlineStr">
@@ -8544,7 +8560,7 @@
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404: No existe la tarjeta 999999 asociada a la cuenta 71</t>
+          <t xml:space="preserve">HTTP 404: No existe la tarjeta 999999 asociada a la cuenta 168</t>
         </is>
       </c>
       <c r="P99" s="8" t="inlineStr">
@@ -8708,7 +8724,7 @@
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">solo se expone **** **** **** 7084</t>
+          <t xml:space="preserve">solo se expone **** **** **** 8809</t>
         </is>
       </c>
       <c r="P101" s="8" t="inlineStr">
@@ -8790,7 +8806,7 @@
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: ids [10, 9, 8]</t>
+          <t xml:space="preserve">HTTP 200: ids [72, 71, 70]</t>
         </is>
       </c>
       <c r="P102" s="8" t="inlineStr">
@@ -9118,7 +9134,7 @@
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: DEPOSIT $250.0 - Ingreso desde tarjeta terminada en 3971</t>
+          <t xml:space="preserve">HTTP 200: DEPOSIT $250.0 - Ingreso desde tarjeta terminada en 1170</t>
         </is>
       </c>
       <c r="P106" s="8" t="inlineStr">
@@ -9200,7 +9216,7 @@
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404: No existe la actividad 999999 en la cuenta 80</t>
+          <t xml:space="preserve">HTTP 404: No existe la actividad 999999 en la cuenta 177</t>
         </is>
       </c>
       <c r="P107" s="8" t="inlineStr">
@@ -10020,7 +10036,7 @@
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">nuevo ingreso 404; el detalle conserva la tarjeta ...6404</t>
+          <t xml:space="preserve">nuevo ingreso 404; el detalle conserva la tarjeta ...2125</t>
         </is>
       </c>
       <c r="P117" s="8" t="inlineStr">
@@ -10439,8 +10455,1402 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-170</t>
+        </is>
+      </c>
+      <c r="B123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir dinero por alias</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con $1.000 de saldo; B registrado.</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con el token de A, POST /accounts/{accountId de A}/transferences con {"destination": alias de B, "amount": 250.50}.</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con el movimiento TRANSFER_OUT y los datos de B (CVU, alias y titular). Saldos: A $749.50, B $250.50.</t>
+        </is>
+      </c>
+      <c r="H123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.transferirPorAliasDevuelve200YMueveElDineroEntreLasDosCuentas</t>
+        </is>
+      </c>
+      <c r="L123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.transferirPorAlias</t>
+        </is>
+      </c>
+      <c r="M123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N123" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O123" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 a Juan Pérez; saldos A=749.5, B=250.5</t>
+        </is>
+      </c>
+      <c r="P123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-171</t>
+        </is>
+      </c>
+      <c r="B124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir dinero por CVU</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con $100; B registrado.</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir $100 a B usando su CVU de 22 dígitos.</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200. A queda en $0 y B en $100.</t>
+        </is>
+      </c>
+      <c r="H124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.transferirPorCvuDevuelve200</t>
+        </is>
+      </c>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.transferirPorCvu</t>
+        </is>
+      </c>
+      <c r="M124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N124" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200; saldos (0.0, 100.0)</t>
+        </is>
+      </c>
+      <c r="P124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-172</t>
+        </is>
+      </c>
+      <c r="B125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fondos insuficientes</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con $100; B registrado.</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir $100.01 a B.</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 410 (fondos insuficientes). Los saldos no cambian.</t>
+        </is>
+      </c>
+      <c r="H125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.sinFondosSuficientesDevuelve410YNoMueveDinero</t>
+        </is>
+      </c>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.fondosInsuficientes</t>
+        </is>
+      </c>
+      <c r="M125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N125" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 410: Fondos insuficientes: el saldo disponible es $100.00</t>
+        </is>
+      </c>
+      <c r="P125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-173</t>
+        </is>
+      </c>
+      <c r="B126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuenta destino inexistente</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con saldo.</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir a un alias inexistente y a un CVU inexistente.</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 (cuenta inexistente) en ambos.</t>
+        </is>
+      </c>
+      <c r="H126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.unaCuentaDestinoInexistenteDevuelve400</t>
+        </is>
+      </c>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.destinoInexistente</t>
+        </is>
+      </c>
+      <c r="M126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N126" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400: La cuenta destino no existe: no.existe.nadie</t>
+        </is>
+      </c>
+      <c r="P126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-174</t>
+        </is>
+      </c>
+      <c r="B127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir a la misma cuenta</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con saldo.</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir a su propio alias.</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400.</t>
+        </is>
+      </c>
+      <c r="H127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.transferirALaMismaCuentaDevuelve400</t>
+        </is>
+      </c>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.mismaCuenta</t>
+        </is>
+      </c>
+      <c r="M127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N127" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400: No se puede transferir a la misma cuenta</t>
+        </is>
+      </c>
+      <c r="P127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-175</t>
+        </is>
+      </c>
+      <c r="B128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir desde una cuenta ajena</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con saldo; B logueado.</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con el token de B, POST /accounts/{accountId de A}/transferences hacia B.</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 403. El saldo de A no cambia.</t>
+        </is>
+      </c>
+      <c r="H128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.noSePuedeTransferirDesdeUnaCuentaAjena</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.cuentaAjena</t>
+        </is>
+      </c>
+      <c r="M128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N128" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 403; saldo de A sin cambios</t>
+        </is>
+      </c>
+      <c r="P128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-176</t>
+        </is>
+      </c>
+      <c r="B129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El destinatario ve la transferencia recibida</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con saldo; B registrado.</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A transfiere $30 a B. B consulta su actividad.</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El primer movimiento de B es TRANSFER_IN (ingreso) con el CVU de A.</t>
+        </is>
+      </c>
+      <c r="H129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.destinatarioVeLaTransferencia</t>
+        </is>
+      </c>
+      <c r="M129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N129" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O129" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B ve TRANSFER_IN de $30.0 desde Juan Pérez</t>
+        </is>
+      </c>
+      <c r="P129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-177</t>
+        </is>
+      </c>
+      <c r="B130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La clave de idempotencia evita transferir dos veces</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con $1.000; B registrado.</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enviar dos veces la misma transferencia de $100 con el mismo header Idempotency-Key.</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ambas HTTP 200 con el mismo id de movimiento; la segunda con Idempotent-Replayed: true. A queda en $900.</t>
+        </is>
+      </c>
+      <c r="H130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.conLaMismaClaveDeIdempotenciaLaTransferenciaSeHaceUnaSolaVez</t>
+        </is>
+      </c>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.idempotencia</t>
+        </is>
+      </c>
+      <c r="M130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N130" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mismo movimiento 107 en ambos envíos; saldo 900.0</t>
+        </is>
+      </c>
+      <c r="P130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-178</t>
+        </is>
+      </c>
+      <c r="B131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montos inválidos en una transferencia</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con $100; B registrado.</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir 0, -1, 1.001 y "10" (texto).</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 en los cuatro casos; el saldo no cambia.</t>
+        </is>
+      </c>
+      <c r="H131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.montosInvalidos</t>
+        </is>
+      </c>
+      <c r="M131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N131" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 400 en los 4 montos; saldo sin cambios</t>
+        </is>
+      </c>
+      <c r="P131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-179</t>
+        </is>
+      </c>
+      <c r="B132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferencias cruzadas simultáneas</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A y B con $1.000 cada uno.</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al mismo tiempo: 10 transferencias de $10 de A a B y 10 de $5 de B a A.</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Las 20 responden 200, sin bloqueos. Saldos finales: A $950 y B $1.050.</t>
+        </is>
+      </c>
+      <c r="H132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borde</t>
+        </is>
+      </c>
+      <c r="I132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.transferenciasCruzadasSimultaneasNoSeBloqueanNiPierdenDinero</t>
+        </is>
+      </c>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N132" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20 respuestas 200; saldos A=950.0, B=1050.0</t>
+        </is>
+      </c>
+      <c r="P132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-180</t>
+        </is>
+      </c>
+      <c r="B133" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Opcional: comprobante y destinatarios</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Últimos destinatarios</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A transfirió a B, luego a C y otra vez a B.</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId de A}/transferences.</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con 2 destinatarios sin repetir: primero B (última transferencia) y después C.</t>
+        </is>
+      </c>
+      <c r="H133" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I133" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J133" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.losUltimosDestinatariosSonLas5CuentasDistintasMasRecientes</t>
+        </is>
+      </c>
+      <c r="L133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.ultimosDestinatarios</t>
+        </is>
+      </c>
+      <c r="M133" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N133" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O133" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200: nacar.maiz.bahia ($2.0), valle.laguna.rama ($1.0)</t>
+        </is>
+      </c>
+      <c r="P133" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-181</t>
+        </is>
+      </c>
+      <c r="B134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Opcional: comprobante y destinatarios</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hasta 5 destinatarios</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A transfirió a 6 cuentas distintas.</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId de A}/transferences.</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con las 5 cuentas más recientes.</t>
+        </is>
+      </c>
+      <c r="H134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borde</t>
+        </is>
+      </c>
+      <c r="I134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.losUltimosDestinatariosSonLas5CuentasDistintasMasRecientes</t>
+        </is>
+      </c>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.destinatariosAjenos</t>
+        </is>
+      </c>
+      <c r="M134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N134" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con las 5 más recientes</t>
+        </is>
+      </c>
+      <c r="P134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-182</t>
+        </is>
+      </c>
+      <c r="B135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Opcional: comprobante y destinatarios</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Destinatarios de una cuenta ajena o sin transferencias</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A y B logueados; A nunca transfirió.</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A consulta sus destinatarios; B consulta los de A.</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A: HTTP 200 con lista vacía. B: HTTP 403.</t>
+        </is>
+      </c>
+      <c r="H135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.sinTransferenciasLaListaDeDestinatariosEstaVaciaYUnaCuentaAjenaDevuelve403</t>
+        </is>
+      </c>
+      <c r="L135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.sinDestinatarios</t>
+        </is>
+      </c>
+      <c r="M135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N135" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O135" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">propia: []; ajena: 403</t>
+        </is>
+      </c>
+      <c r="P135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-183</t>
+        </is>
+      </c>
+      <c r="B136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reutilizar la clave de idempotencia con otros datos</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con $1.000; B registrado.</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir $100 con Idempotency-Key = K. Luego transferir $1 con la misma clave K.</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La primera: HTTP 200. La segunda: HTTP 409 (la clave ya se usó para otra operación). A queda en $900.</t>
+        </is>
+      </c>
+      <c r="H136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.reutilizarLaClaveConOtrosDatosDevuelve409</t>
+        </is>
+      </c>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.claveReutilizada</t>
+        </is>
+      </c>
+      <c r="M136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N136" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O136" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 409: La clave Idempotency-Key ya se usó para una operación con otros datos</t>
+        </is>
+      </c>
+      <c r="P136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-184</t>
+        </is>
+      </c>
+      <c r="B137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CVU pegado con espacios o guiones</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con saldo; B registrado.</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir usando el CVU de B con un espacio y un guion en el medio.</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200: el CVU se reconoce.</t>
+        </is>
+      </c>
+      <c r="H137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borde</t>
+        </is>
+      </c>
+      <c r="I137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja</t>
+        </is>
+      </c>
+      <c r="J137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.unCvuConEspaciosOGuionesSeReconoce</t>
+        </is>
+      </c>
+      <c r="L137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.cvuConEspacios</t>
+        </is>
+      </c>
+      <c r="M137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N137" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con destino "80382644 0129840-7591067"</t>
+        </is>
+      </c>
+      <c r="P137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-190</t>
+        </is>
+      </c>
+      <c r="B138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Opcional: comprobante y destinatarios</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descargar el comprobante en PDF</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A transfirió $40 a B.</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId}/activity/{id}/receipt.</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200, Content-Type application/pdf, descarga como comprobante-{id}.pdf con los datos del detalle.</t>
+        </is>
+      </c>
+      <c r="H138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.elComprobanteEsUnPdfDescargable</t>
+        </is>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.comprobantePdf</t>
+        </is>
+      </c>
+      <c r="M138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N138" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O138" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 application/pdf, 1 KB, attachment; filename="comprobante-179.pdf"</t>
+        </is>
+      </c>
+      <c r="P138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-191</t>
+        </is>
+      </c>
+      <c r="B139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Opcional: comprobante y destinatarios</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comprobante de un movimiento ajeno</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A transfirió a B.</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B pide el comprobante del movimiento de A usando la cuenta de B.</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 404 en JSON (no un PDF).</t>
+        </is>
+      </c>
+      <c r="H139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguridad</t>
+        </is>
+      </c>
+      <c r="I139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="J139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regresión</t>
+        </is>
+      </c>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.elComprobanteDeUnMovimientoAjenoNoSePuedeDescargar</t>
+        </is>
+      </c>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.comprobanteAjeno</t>
+        </is>
+      </c>
+      <c r="M139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N139" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 404: No existe la actividad 182 en la cuenta 233</t>
+        </is>
+      </c>
+      <c r="P139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P122"/>
+  <autoFilter ref="A1:P139"/>
 </worksheet>
 </file>
 
@@ -10620,7 +12030,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201, id=1, cvu=6334344006712411812213, alias=condor.relampago.laguna</t>
+          <t xml:space="preserve">HTTP 201, id=98, cvu=3257469782009407052174, alias=roca.delta.agua</t>
         </is>
       </c>
       <c r="P2" s="8" t="inlineStr">
@@ -10784,7 +12194,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: Juan Pérez &lt;qa584n34@mail.com&gt;</t>
+          <t xml:space="preserve">HTTP 200: Juan Pérez &lt;qa439n34@mail.com&gt;</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -11269,19 +12679,19 @@
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bloqueado</t>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se pudo ejecutar: en esta máquina Docker Desktop no arranca porque Windows no tiene habilitada la característica "Plataforma de máquina virtual" (requiere administrador y reinicio). docker compose config valida el archivo.</t>
+          <t xml:space="preserve">Ejecutado en GitHub Actions (job docker-e2e, CI #4, commit 08442ee): docker compose up -d --build levantó MySQL, MailHog y los 5 servicios; los 4 servicios quedaron UP en Eureka y la automatización RestAssured (75 de 75) y la suite de casos pasaron contra MySQL y MailHog.</t>
         </is>
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">02/10/2026</t>
+          <t xml:space="preserve">15/10/2026</t>
         </is>
       </c>
     </row>
@@ -11358,7 +12768,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: cvu=9412470896288656923251, alias=pasto.remo.tero, balance=0.0</t>
+          <t xml:space="preserve">HTTP 200: cvu=9713684828224062434639, alias=pradera.perla.trueno, balance=0.0</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
@@ -11440,7 +12850,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">usuario Juan Pérez; cvu=7356793963469973822129, alias=fogata.avion.glaciar</t>
+          <t xml:space="preserve">usuario Juan Pérez; cvu=6658065001634942495360, alias=tigre.yaguarete.remo</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
@@ -11604,7 +13014,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: alias=nuevo.alias.qa56</t>
+          <t xml:space="preserve">HTTP 200: alias=nuevo.alias.qa153</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
@@ -11686,7 +13096,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 201: VISA **** **** **** 0085, tipo DEBIT</t>
+          <t xml:space="preserve">HTTP 201: VISA **** **** **** 4931, tipo DEBIT</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
@@ -11932,7 +13342,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: ids [10, 9, 8]</t>
+          <t xml:space="preserve">HTTP 200: ids [72, 71, 70]</t>
         </is>
       </c>
       <c r="P18" s="8" t="inlineStr">
@@ -12014,7 +13424,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 200: DEPOSIT $250.0 - Ingreso desde tarjeta terminada en 3971</t>
+          <t xml:space="preserve">HTTP 200: DEPOSIT $250.0 - Ingreso desde tarjeta terminada en 1170</t>
         </is>
       </c>
       <c r="P19" s="8" t="inlineStr">
@@ -12105,7 +13515,253 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-170</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir dinero por alias</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con $1.000 de saldo; B registrado.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con el token de A, POST /accounts/{accountId de A}/transferences con {"destination": alias de B, "amount": 250.50}.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con el movimiento TRANSFER_OUT y los datos de B (CVU, alias y titular). Saldos: A $749.50, B $250.50.</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.transferirPorAliasDevuelve200YMueveElDineroEntreLasDosCuentas</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.transferirPorAlias</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 a Juan Pérez; saldos A=749.5, B=250.5</t>
+        </is>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-172</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Transferir dinero</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fondos insuficientes</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A con $100; B registrado.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transferir $100.01 a B.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 410 (fondos insuficientes). Los saldos no cambian.</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negativo</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.sinFondosSuficientesDevuelve410YNoMueveDinero</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.fondosInsuficientes</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 410: Fondos insuficientes: el saldo disponible es $100.00</t>
+        </is>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-180</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 Opcional: comprobante y destinatarios</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Últimos destinatarios</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A transfirió a B, luego a C y otra vez a B.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /accounts/{accountId de A}/transferences.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 con 2 destinatarios sin repetir: primero B (última transferencia) y después C.</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivo</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smoke + Regresión</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint4ApiTest.losUltimosDestinatariosSonLas5CuentasDistintasMasRecientes</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TransferApiTest.ultimosDestinatarios</t>
+        </is>
+      </c>
+      <c r="M23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Script</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pasó</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200: nacar.maiz.bahia ($2.0), valle.laguna.rama ($1.0)</t>
+        </is>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P20"/>
+  <autoFilter ref="A1:P23"/>
 </worksheet>
 </file>
</xml_diff>